<commit_message>
Update: Integration with Kaggle and data cleaning
</commit_message>
<xml_diff>
--- a/df_26.xlsx
+++ b/df_26.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Cruzeiro Saf</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -642,30 +642,30 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>20005</v>
+        <v>20007</v>
       </c>
       <c r="C5" t="n">
         <v>1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Coritiba S.a.f.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -691,7 +691,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>20014</v>
+        <v>20385</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
@@ -703,7 +703,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Mirassol</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -714,7 +714,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Grêmio</t>
+          <t>Vasco da Gama Saf</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -740,7 +740,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>20385</v>
+        <v>20005</v>
       </c>
       <c r="C7" t="n">
         <v>1</v>
@@ -752,7 +752,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -763,7 +763,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Vasco da Gama Saf</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -789,19 +789,19 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>61377</v>
+        <v>20014</v>
       </c>
       <c r="C8" t="n">
         <v>1</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -812,7 +812,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Grêmio</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -838,7 +838,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>20052</v>
+        <v>61377</v>
       </c>
       <c r="C9" t="n">
         <v>1</v>
@@ -850,18 +850,18 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Athletico Paranaense</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Internacional</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -887,7 +887,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>20007</v>
+        <v>20052</v>
       </c>
       <c r="C10" t="n">
         <v>1</v>
@@ -899,7 +899,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Athletico Paranaense</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -910,7 +910,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Coritiba S.a.f.</t>
+          <t>Internacional</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Atlético Mineiro Saf</t>
+          <t>Atlético Mineiro</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -992,12 +992,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Atlético Mineiro Saf</t>
+          <t>Palmeiras</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Palmeiras</t>
+          <t>Atlético Mineiro</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1034,7 +1034,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>60646</v>
+        <v>20013</v>
       </c>
       <c r="C13" t="n">
         <v>1</v>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Vasco da Gama Saf</t>
+          <t>Grêmio</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Mirassol</t>
+          <t>Fluminense</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1083,30 +1083,30 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>20013</v>
+        <v>61590</v>
       </c>
       <c r="C14" t="n">
         <v>1</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Grêmio</t>
+          <t>Coritiba S.a.f.</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Fluminense</t>
+          <t>Red Bull Bragantino</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1132,19 +1132,19 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>20001</v>
+        <v>60646</v>
       </c>
       <c r="C15" t="n">
         <v>1</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Corinthians</t>
+          <t>Vasco da Gama Saf</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Mirassol</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1279,7 +1279,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>61590</v>
+        <v>20001</v>
       </c>
       <c r="C18" t="n">
         <v>1</v>
@@ -1291,18 +1291,18 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Coritiba S.a.f.</t>
+          <t>Corinthians</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Red Bull Bragantino</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Cruzeiro Saf</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -1468,6 +1468,888 @@
       </c>
       <c r="M21" t="n">
         <v>20</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="n">
+        <v>20007</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Red Bull Bragantino</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Atlético Mineiro</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>6</v>
+      </c>
+      <c r="K22" t="n">
+        <v>2</v>
+      </c>
+      <c r="L22" t="n">
+        <v>2</v>
+      </c>
+      <c r="M22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="n">
+        <v>20002</v>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Palmeiras</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>4</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1</v>
+      </c>
+      <c r="L23" t="n">
+        <v>4</v>
+      </c>
+      <c r="M23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="n">
+        <v>20086</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Chapecoense</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Vasco da Gama Saf</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>4</v>
+      </c>
+      <c r="K24" t="n">
+        <v>1</v>
+      </c>
+      <c r="L24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="n">
+        <v>20385</v>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Mirassol</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Remo</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>4</v>
+      </c>
+      <c r="K25" t="n">
+        <v>1</v>
+      </c>
+      <c r="L25" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="n">
+        <v>20005</v>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Santos Fc</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>4</v>
+      </c>
+      <c r="K26" t="n">
+        <v>1</v>
+      </c>
+      <c r="L26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M26" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="n">
+        <v>20014</v>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Fluminense</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Bahia</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>4</v>
+      </c>
+      <c r="K27" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" t="n">
+        <v>1</v>
+      </c>
+      <c r="M27" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="n">
+        <v>61377</v>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Bahia</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Fluminense</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>4</v>
+      </c>
+      <c r="K28" t="n">
+        <v>1</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1</v>
+      </c>
+      <c r="M28" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="n">
+        <v>60175</v>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Botafogo</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>3</v>
+      </c>
+      <c r="G29" t="n">
+        <v>5</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Grêmio</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>3</v>
+      </c>
+      <c r="K29" t="n">
+        <v>1</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="n">
+        <v>20013</v>
+      </c>
+      <c r="C30" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Grêmio</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>5</v>
+      </c>
+      <c r="G30" t="n">
+        <v>3</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Botafogo</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1</v>
+      </c>
+      <c r="L30" t="n">
+        <v>1</v>
+      </c>
+      <c r="M30" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>61590</v>
+      </c>
+      <c r="C31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Coritiba S.a.f.</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Cruzeiro</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>3</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>20018</v>
+      </c>
+      <c r="C32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>5</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Palmeiras</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>3</v>
+      </c>
+      <c r="K32" t="n">
+        <v>1</v>
+      </c>
+      <c r="L32" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M32" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>59849</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Coritiba S.a.f.</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Cruzeiro</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>3</v>
+      </c>
+      <c r="K33" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" t="n">
+        <v>-3</v>
+      </c>
+      <c r="M33" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>60646</v>
+      </c>
+      <c r="C34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Vasco da Gama Saf</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Chapecoense</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" t="n">
+        <v>-1</v>
+      </c>
+      <c r="M34" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>20016</v>
+      </c>
+      <c r="C35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>-1</v>
+      </c>
+      <c r="M35" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="n">
+        <v>62194</v>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Atlético Mineiro</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Red Bull Bragantino</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>1</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>-1</v>
+      </c>
+      <c r="M36" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="n">
+        <v>20011</v>
+      </c>
+      <c r="C37" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Internacional</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>-1</v>
+      </c>
+      <c r="M37" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>20008</v>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Santos Fc</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M38" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>20022</v>
+      </c>
+      <c r="C39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Remo</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>2</v>
+      </c>
+      <c r="G39" t="n">
+        <v>2</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Mirassol</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="n">
+        <v>-2</v>
+      </c>
+      <c r="M39" t="n">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>